<commit_message>
Add Waste Expo 2026 WasteVantage invite email template
Outreach email inviting Melbourne waste operators to visit
WasteVantage at Waste Expo Australia (28–29 Oct 2026, MCEC),
covering product benefits for skip, rearlift and garden bag
operators, plus a short follow-up version.

Co-authored-by: hendrikdamai-art <hendrik.damai@gmail.com>
</commit_message>
<xml_diff>
--- a/research/Melbourne_Waste_Skip_Rearlift_GardenBag_Companies.xlsx
+++ b/research/Melbourne_Waste_Skip_Rearlift_GardenBag_Companies.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Melbourne Waste Companies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Research Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Invite Email Template" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Research Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Melbourne Waste Companies'!$A$1:$K$60</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +38,20 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -88,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -103,6 +118,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3798,6 +3819,222 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Waste Expo Australia 2026 — WasteVantage invite email</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Waste Expo Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>28 – 29 October 2026, 9am – 5pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Venue</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Melbourne Convention and Exhibition Centre (MCEC), South Wharf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Expo website</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.wasteexpoaustralia.com.au/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>WasteVantage</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://ihublogistics.com/wastevantage/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>SUBJECT (option 1)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>{{Company Name}} — meet WasteVantage at Waste Expo Australia (28–29 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>SUBJECT (option 2)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Invitation: see WasteVantage live at Waste Expo Melbourne, 28–29 October</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>EMAIL BODY — copy below</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="520" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hi {{First Name / team at Company Name}},
+We're writing from WasteVantage to invite you to visit us at Waste Expo Australia 2026.
+When: Wednesday 28 – Thursday 29 October 2026, 9am–5pm
+Where: Melbourne Convention and Exhibition Centre (MCEC)
+Event: https://www.wasteexpoaustralia.com.au/
+Waste Expo is Australia's leading gathering for waste, recycling and resource recovery — with 3,500+ attendees, 140+ exhibitors and free education sessions. It's the best place this year to see what's next for operators like yours.
+WHY VISIT WASTEVANTAGE AT THE EXPO?
+WasteVantage is purpose-built waste management software for Australian and New Zealand operators — including skip bin hire, rearlift / wheelie bin rounds, front lift, and garden / skip bag style services.
+At our stand you can:
+• See a live demo of bookings, dispatch, bin tracking and driver run sheets in one system
+• Talk through your operation (skip delivery/pickup, rearlift schedules, garden bag collections) with people who understand the workflow
+• Compare how you run today vs automating pricing, job scheduling, customer SMS and same-day invoicing
+• Ask about Xero / MYOB / Stripe integrations so office admin and cash flow stay connected
+• Get a clear view of whether WasteVantage fits a single-stream business or a multi-stream fleet (skips + rearlift + bags)
+WHAT WASTEVANTAGE CAN DO FOR {{Company Name}}
+If you're juggling phone bookings, spreadsheets, drivers and invoices, the expo is a low-risk way to see how operators are cutting admin and missed jobs:
+• High volume skip deliveries, pickups and swaps → Smart scheduling &amp; dispatch so jobs aren't missed or double-booked
+• "Where is that bin?" / lost assets → Real-time bin status, location and customer tracking
+• Drivers needing paper run sheets and constant office calls → Automated run sheets on driver phones + live job updates
+• Slow or messy invoicing after jobs close → One-click / same-day invoicing synced to Xero or MYOB
+• Customers chasing ETAs → Automated SMS / notifications and clearer service proof
+• Growing into rearlift or garden bags alongside skips → One platform for multi-stream operations
+Built and supported in Australia for local operators — not a generic overseas logistics tool bolted onto waste.
+WHY COME IN PERSON?
+• Free trade visitor registration for industry professionals via the expo site
+• Face-to-face demo beats a cold website click — bring your toughest operational question
+• See peers and suppliers in one venue while you're there
+• Melbourne timing — ideal if you already service metro Melbourne and surrounds
+If you're free on either day, we'd love 15–20 minutes at our stand to walk you through a demo tailored to skip / rearlift / garden bag work.
+RSVP / book a time: reply to this email with a preferred day (28 or 29 Oct) and we'll hold a slot for {{Company Name}}.
+Expo info &amp; visitor registration: https://www.wasteexpoaustralia.com.au/
+Learn more about WasteVantage: https://ihublogistics.com/wastevantage/
+Looking forward to meeting you in Melbourne.
+Kind regards,
+{{Your Name}}
+{{Your Title}}
+WasteVantage
+{{Your Phone}}
+{{Your Email}}
+https://ihublogistics.com/wastevantage/
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>SHORT FOLLOW-UP SUBJECT</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Quick reminder — WasteVantage at Waste Expo (28–29 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>SHORT FOLLOW-UP BODY</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="160" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Hi {{First Name}},
+Just a short follow-up on our invite to meet at Waste Expo Australia, 28–29 October 2026 at MCEC Melbourne.
+We'll be showing WasteVantage live — bookings, bin tracking, driver apps and automated invoicing for skip, rearlift and garden bag operators.
+If you're attending, reply with your preferred day and we'll book a 15-minute demo for {{Company Name}}.
+Expo: https://www.wasteexpoaustralia.com.au/
+Thanks,
+{{Your Name}} | WasteVantage</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>SENDING TIPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>1. Replace {{Company Name}} / {{First Name}} from the company list sheet.  2. Add booth/stand number once confirmed.  3. Send one-to-one (not bulk BCC).  4. Confirm exhibitor registration &amp; free visitor entry before promising it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A12:B12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Enrich waste company list with 13 newly found public emails
Filled yellow-cell rows where contact emails were published on
company sites or directories (now 51/59 have emails). Remaining
8 only publish phone/forms. Refreshed CSV export.

Co-authored-by: hendrikdamai-art <hendrik.damai@gmail.com>
</commit_message>
<xml_diff>
--- a/research/Melbourne_Waste_Skip_Rearlift_GardenBag_Companies.xlsx
+++ b/research/Melbourne_Waste_Skip_Rearlift_GardenBag_Companies.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Melbourne Waste Companies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Invite Email Template" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Research Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Melbourne Waste Companies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invite Email Template" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Melbourne Waste Companies'!$A$1:$K$60</definedName>
@@ -54,7 +54,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -122,6 +127,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1071,9 +1079,9 @@
           <t>03 9460 5333</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Not published clearly (see website)</t>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>admin@unlimitedbins.com.au</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1108,7 +1116,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Also unlimitedbins.com.au; email obfuscated on site</t>
+          <t>Email from company contact page / privacy policy | was: Also unlimitedbins.com.au; email obfuscated on site</t>
         </is>
       </c>
     </row>
@@ -1181,9 +1189,9 @@
           <t>03 9005 7675</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Not found publicly (call/book online)</t>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>info@choicebins.com.au</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1218,7 +1226,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Company website; email not listed</t>
+          <t>Email from company contact page | was: Company website; email not listed</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1721,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Company website</t>
+          <t>No public email found after deep search; phone/office only (03 8872 7879)</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1776,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Company site; CoM waste providers list</t>
+          <t>No public general email found; use phone 1300 219 001 or online form</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2161,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Company website; CoM list</t>
+          <t>No public email found; phone only 03 9824 1975</t>
         </is>
       </c>
     </row>
@@ -2391,9 +2399,9 @@
           <t>1300 550 408</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Not published (contact form)</t>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>contact@wastewise.com.au</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -2428,7 +2436,7 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Company contact page; CoM list</t>
+          <t>Also sales@wastewise.com.au on older site page | was: Company contact page; CoM list</t>
         </is>
       </c>
     </row>
@@ -2501,9 +2509,9 @@
           <t>1300 586 548</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Not published (online booking / form)</t>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>info@aussieskipbags.com.au</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -2538,7 +2546,7 @@
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>Also collects Croc Bags; company site</t>
+          <t>Also operations@aussieskipbags.com.au | was: Also collects Croc Bags; company site</t>
         </is>
       </c>
     </row>
@@ -2703,7 +2711,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Melbourne office (03) 8397 5100; CoM list</t>
+          <t>No public general email; use 13 13 39 or online enquiry form</t>
         </is>
       </c>
     </row>
@@ -2721,9 +2729,9 @@
           <t>13 29 55</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Not published (online enquiry form)</t>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>cx.service@anz.veolia.com</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -2758,7 +2766,7 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>CoM waste providers list</t>
+          <t>Customer experience team email from Veolia ANZ portals page; also call 13 29 55 | was: CoM waste providers list</t>
         </is>
       </c>
     </row>
@@ -2831,9 +2839,9 @@
           <t>13 15 46</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Not published nationally (franchise local)</t>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>jimscontracts@jims.net</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2868,7 +2876,7 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Franchise model; local franchisees vary</t>
+          <t>Jim's Contracts / national office email; local franchisees may differ — also call 13 15 46 | was: Franchise model; local franchisees vary</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3206,7 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Connects to local operators</t>
+          <t>Referral aggregator — no public email on site; phone 0482 392 415</t>
         </is>
       </c>
     </row>
@@ -3216,14 +3224,14 @@
           <t>03 9670 4042</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Not found publicly (call)</t>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>admin@phoenixwastecollection.com.au</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Search company name + Melbourne</t>
+          <t>https://www.phoenixwastecollection.com.au/</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3253,7 +3261,7 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>City of Melbourne waste providers list</t>
+          <t>Company contact page; also phone 03 9670 4042 | was: City of Melbourne waste providers list</t>
         </is>
       </c>
     </row>
@@ -3271,44 +3279,44 @@
           <t>1300 292 783</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Not found publicly (call)</t>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>sales@awaste.com.au</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Search company name + Melbourne</t>
+          <t>https://www.australianwastemanagement.com.au/</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
+          <t>56 Paraweena Drive, Truganina VIC 3029</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Yes (listed)</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Yes (listed recycling streams)</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Check with company</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
           <t>Melbourne</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>Yes (listed)</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr">
-        <is>
-          <t>Yes (listed recycling streams)</t>
-        </is>
-      </c>
-      <c r="I51" s="3" t="inlineStr">
-        <is>
-          <t>Check with company</t>
-        </is>
-      </c>
-      <c r="J51" s="3" t="inlineStr">
-        <is>
-          <t>Melbourne</t>
-        </is>
-      </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>City of Melbourne waste providers list</t>
+          <t>Also known as AWASTE; Wyndham directory + company site | was: City of Melbourne waste providers list</t>
         </is>
       </c>
     </row>
@@ -3323,22 +3331,22 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>1300 267 469</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Not found publicly (call)</t>
+          <t>1300 267 4696</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>contactcentre@coriowm.com.au</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Search company name + Geelong/Melbourne</t>
+          <t>https://www.coriowm.com.au/</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Geelong / Melbourne region</t>
+          <t>41-49 Wills Cres, Moolap VIC 3224 (also Altona North &amp; Dandenong South)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -3363,7 +3371,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>CoM list (phone shown as 1300 267 4696 on CoM; verify digit count)</t>
+          <t>Also sales@coriowm.com.au; serves Geelong, Ballarat &amp; Melbourne | was: CoM list (phone shown as 1300 267 4696 on CoM; verify digit count)</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3426,7 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>City of Melbourne waste providers list</t>
+          <t>Brand largely under Veolia; use 131 335 / Veolia channels; no separate public email found</t>
         </is>
       </c>
     </row>
@@ -3436,44 +3444,44 @@
           <t>1300 723 232</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Not found publicly (call)</t>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>info@waynecleaningsystems.com.au</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Search Wayne Cleaning Systems waste Melbourne</t>
+          <t>https://www.waynecleaningsystems.com.au/</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
+          <t>147 Miller Street / 23 Taylor Street, Thornbury VIC; Waste depot 10 Wentworth Ct, Thomastown</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Listed provider</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Yes (listed streams)</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Check with company</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
           <t>Melbourne</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>Listed provider</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>Yes (listed streams)</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>Check with company</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>Melbourne</t>
-        </is>
-      </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>City of Melbourne waste providers list</t>
+          <t>Company website contact | was: City of Melbourne waste providers list</t>
         </is>
       </c>
     </row>
@@ -3491,9 +3499,9 @@
           <t>1300 954 576</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>Not found publicly (call)</t>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>peter@limitlessrecycling.com.au</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -3503,32 +3511,32 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
+          <t>33 Malua Street, Reservoir VIC</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Listed provider</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Yes (listed)</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Check with company</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
           <t>Melbourne</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>Listed provider</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>Yes (listed)</t>
-        </is>
-      </c>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>Check with company</t>
-        </is>
-      </c>
-      <c r="J55" s="3" t="inlineStr">
-        <is>
-          <t>Melbourne</t>
-        </is>
-      </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>City of Melbourne waste providers list</t>
+          <t>Recycling Near You directory listing | was: City of Melbourne waste providers list</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3591,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>City of Melbourne waste providers list</t>
+          <t>No public email found; phone only 0406 267 275</t>
         </is>
       </c>
     </row>
@@ -3601,14 +3609,14 @@
           <t>0452 458 909</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>Not found publicly (call)</t>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>estimatorvic@aldcorporate.com.au</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Search Expert Demo waste Melbourne</t>
+          <t>https://www.expertdemo.com.au/</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -3638,7 +3646,7 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>City of Melbourne construction waste providers</t>
+          <t>Expert Demo site lists ALD Corporate VIC estimator email — confirm before outreach; phone 0452 458 909 from CoM list | was: City of Melbourne construction waste providers</t>
         </is>
       </c>
     </row>
@@ -3663,7 +3671,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Search Revert Group Melbourne waste</t>
+          <t>https://revertgroup.com.au/</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3693,7 +3701,7 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>City of Melbourne construction waste providers</t>
+          <t>No public email on site; phone 1300 307 450 / 0416 416 224 or online form — https://revertgroup.com.au/</t>
         </is>
       </c>
     </row>
@@ -3711,44 +3719,44 @@
           <t>1300 648 088</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>Not found publicly (call)</t>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>info@wasteninja.com.au</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Search Waste Ninja Melbourne</t>
+          <t>https://wasteninja.com.au/</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
+          <t>5A Connection Drive, Campbellfield VIC 3061</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Check with company</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Check with company</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Food organics (listed)</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
           <t>Melbourne</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>Check with company</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>Check with company</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>Food organics (listed)</t>
-        </is>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>Melbourne</t>
-        </is>
-      </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>City of Melbourne food organics providers</t>
+          <t>Company contact page | was: City of Melbourne food organics providers</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -4078,7 +4086,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -4158,6 +4166,181 @@
       <c r="A18" t="inlineStr">
         <is>
           <t>- This list is for research/outreach; not an endorsement. Verify details before use as contacts change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Email enrichment update</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Newly filled emails: 13; still missing public email: 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Unlimited Bins (Skip Hire Melbourne)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>admin@unlimitedbins.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Choice Bins</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>info@choicebins.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Waste Wise Environmental</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>contact@wastewise.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Aussie Skip Bags</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>info@aussieskipbags.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Veolia Environmental Services</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>cx.service@anz.veolia.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Jim's Skip Bins</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>jimscontracts@jims.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Phoenix Environmental Waste</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>admin@phoenixwastecollection.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Australian Waste Management</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>sales@awaste.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Corio Waste Management</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>contactcentre@coriowm.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Wayne Cleaning Systems</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>info@waynecleaningsystems.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Limitless Secure Recycling &amp; Waste Solutions</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>peter@limitlessrecycling.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Expert Demo</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>estimatorvic@aldcorporate.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Waste Ninja</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>info@wasteninja.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Green email cells = newly found in this enrichment pass. Yellow = still no public email (use phone).</t>
         </is>
       </c>
     </row>

</xml_diff>